<commit_message>
Updated Excel - 19 August 2026
</commit_message>
<xml_diff>
--- a/vaibhav.xlsx
+++ b/vaibhav.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F376A7E-3713-4690-B31E-06C30B65D02A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F3C4FB7-9A6F-4FAF-AB61-95976C636E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -233,6 +233,24 @@
   </si>
   <si>
     <t>classes took most of the time</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>classes were minimum today</t>
+  </si>
+  <si>
+    <t>nil</t>
+  </si>
+  <si>
+    <t>5o</t>
+  </si>
+  <si>
+    <t>Very Unsatisfied</t>
   </si>
 </sst>
 </file>
@@ -1199,126 +1217,222 @@
       <c r="A10" s="13">
         <v>46247</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+      <c r="B10" s="14">
+        <v>410</v>
+      </c>
+      <c r="C10" s="14">
+        <v>60</v>
+      </c>
+      <c r="D10" s="14">
+        <v>180</v>
+      </c>
+      <c r="E10" s="14">
+        <v>0</v>
+      </c>
+      <c r="F10" s="14">
+        <v>250</v>
+      </c>
+      <c r="G10" s="14">
+        <v>3</v>
+      </c>
+      <c r="H10" s="14">
+        <v>180</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>360</v>
       </c>
       <c r="K10" s="16" t="s">
         <v>64</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="M10" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="N10" s="17"/>
+      <c r="N10" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+      <c r="B11" s="14">
+        <v>440</v>
+      </c>
+      <c r="C11" s="14">
+        <v>30</v>
+      </c>
+      <c r="D11" s="14">
+        <v>90</v>
+      </c>
+      <c r="E11" s="14">
+        <v>70</v>
+      </c>
+      <c r="F11" s="14">
+        <v>200</v>
+      </c>
+      <c r="G11" s="14">
+        <v>4</v>
+      </c>
+      <c r="H11" s="14">
+        <v>140</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
+        <v>470</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>59</v>
+      </c>
       <c r="N11" s="17"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
         <v>46249</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+      <c r="B12" s="14">
+        <v>520</v>
+      </c>
+      <c r="C12" s="14">
+        <v>90</v>
+      </c>
+      <c r="D12" s="14">
+        <v>240</v>
+      </c>
+      <c r="E12" s="14">
+        <v>120</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" s="14">
+        <v>180</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
+        <v>290</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N12" s="17"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>46250</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="B13" s="14">
+        <v>600</v>
+      </c>
+      <c r="C13" s="14">
+        <v>90</v>
+      </c>
+      <c r="D13" s="14">
+        <v>200</v>
+      </c>
+      <c r="E13" s="14">
+        <v>70</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="14">
+        <v>240</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
+        <v>240</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N13" s="17"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
         <v>46251</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="B14" s="14">
+        <v>305</v>
+      </c>
+      <c r="C14" s="14">
+        <v>10</v>
+      </c>
+      <c r="D14" s="14">
+        <v>150</v>
+      </c>
+      <c r="E14" s="14">
+        <v>60</v>
+      </c>
+      <c r="F14" s="14">
+        <v>300</v>
+      </c>
+      <c r="G14" s="14">
+        <v>6</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>825</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
+        <v>615</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1328,33 +1442,55 @@
       <c r="B15" s="14">
         <v>210</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
+      <c r="C15" s="14">
+        <v>0</v>
+      </c>
+      <c r="D15" s="14">
+        <v>80</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>350</v>
+      </c>
+      <c r="G15" s="14">
+        <v>7</v>
+      </c>
+      <c r="H15" s="14">
+        <v>40</v>
+      </c>
       <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v>210</v>
+        <v>680</v>
       </c>
       <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v>1230</v>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+        <v>760</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
+      <c r="A16" s="13">
+        <v>46253</v>
+      </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
+      <c r="G16" s="14">
+        <v>7</v>
+      </c>
       <c r="H16" s="14"/>
       <c r="I16" s="15" t="str">
         <f t="shared" si="0"/>
@@ -1370,13 +1506,17 @@
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
+      <c r="A17" s="13">
+        <v>46254</v>
+      </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
+      <c r="G17" s="14">
+        <v>3</v>
+      </c>
       <c r="H17" s="14"/>
       <c r="I17" s="15" t="str">
         <f t="shared" si="0"/>
@@ -1392,13 +1532,17 @@
       <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
+      <c r="A18" s="13">
+        <v>46255</v>
+      </c>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="G18" s="14">
+        <v>4</v>
+      </c>
       <c r="H18" s="14"/>
       <c r="I18" s="15" t="str">
         <f t="shared" si="0"/>

</xml_diff>